<commit_message>
fix: Similarity around amdt body was not filtered properly
</commit_message>
<xml_diff>
--- a/tests/integration/test_data/test_similarities_expose.xlsx
+++ b/tests/integration/test_data/test_similarities_expose.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10112"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/amendements-intelligents/tests/integration/test_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/graal/tests/integration/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BA0ECDB-0AA8-8D4D-93A4-75A51962DC10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6828E34D-8B56-574A-BC39-ABB0D5A17FA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="34400" windowHeight="28300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vieux amendements" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="113">
   <si>
     <t>Num amdt</t>
   </si>
@@ -391,17 +391,26 @@
     <t>origin_project</t>
   </si>
   <si>
-    <t>PLFSS</t>
+    <t>PLFSS 2024</t>
   </si>
   <si>
-    <t>Réponse copiée de : PLFSS 2024
+    <t>PLFSS 2023</t>
+  </si>
+  <si>
+    <t>PLFSS 2022</t>
+  </si>
+  <si>
+    <t>PLACSS 2021</t>
+  </si>
+  <si>
+    <t>Réponse copiée de : PLFSS 2023
 Numéro d'amendement : 2
 Lecture : an 16
 Organe : Organe456
 Colonne similaire : Exposé amdt</t>
   </si>
   <si>
-    <t>Réponse copiée de : PLFSS 2024
+    <t>Réponse copiée de : PLFSS 2022
 Numéro d'amendement : 15638
 Lecture : an 16
 Organe : PO791932
@@ -409,22 +418,22 @@
 Sort copié : Irrecevable</t>
   </si>
   <si>
-    <t>Réponse copiée de : PLFSS 2022
-Numéro d'amendement : 23
+    <t>Réponse copiée de : PLACSS 2021
+Numéro d'amendement : 4
 Lecture : an 16
-Organe : PO791932
+Organe : Organe456
 Colonne similaire : Exposé amdt</t>
   </si>
   <si>
-    <t>Réponse copiée de : PLFSS 2022
-Numéro d'amendement : 19416
-Lecture : an 16
+    <t>Réponse copiée de : PLFSS 2023
+Numéro d'amendement : 5726
+Lecture : senat 16
 Organe : PO78718
 Colonne similaire : Exposé amdt</t>
   </si>
   <si>
-    <t>Réponse copiée de : PLFSS 2022
-Numéro d'amendement : 146
+    <t>Réponse copiée de : PLFSS 2024
+Numéro d'amendement : 20502
 Lecture : an 16
 Organe : PO791932
 Colonne similaire : Exposé amdt
@@ -432,28 +441,25 @@
   </si>
   <si>
     <t>Réponse copiée de : PLFSS 2023
-Numéro d'amendement : 20502
+Numéro d'amendement : 19416
+Lecture : an 16
+Organe : PO78718
+Colonne similaire : Exposé amdt</t>
+  </si>
+  <si>
+    <t>Réponse copiée de : PLFSS 2024
+Numéro d'amendement : 23
+Lecture : an 16
+Organe : PO791932
+Colonne similaire : Exposé amdt</t>
+  </si>
+  <si>
+    <t>Réponse copiée de : PLFSS 2024
+Numéro d'amendement : 146
 Lecture : an 16
 Organe : PO791932
 Colonne similaire : Exposé amdt
 Sort copié : Irrecevable</t>
-  </si>
-  <si>
-    <t>Réponse copiée de : PLFSS 2022
-Numéro d'amendement : 5726
-Lecture : senat 16
-Organe : PO78718
-Colonne similaire : Exposé amdt</t>
-  </si>
-  <si>
-    <t>PLACSS</t>
-  </si>
-  <si>
-    <t>Réponse copiée de : PLACSS 2023
-Numéro d'amendement : 4
-Lecture : an 16
-Organe : Organe456
-Colonne similaire : Exposé amdt</t>
   </si>
 </sst>
 </file>
@@ -475,21 +481,25 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -922,7 +932,7 @@
     </row>
     <row r="3" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B3" s="6">
         <v>2</v>
@@ -955,7 +965,7 @@
     </row>
     <row r="4" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="18" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B4" s="9">
         <v>15638</v>
@@ -987,7 +997,7 @@
     </row>
     <row r="5" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B5" s="9">
         <v>16464</v>
@@ -1051,7 +1061,7 @@
     </row>
     <row r="7" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B7" s="9">
         <v>19416</v>
@@ -1115,7 +1125,7 @@
     </row>
     <row r="9" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B9" s="9">
         <v>16634</v>
@@ -1179,7 +1189,7 @@
     </row>
     <row r="11" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B11" s="9">
         <v>19412</v>
@@ -1275,7 +1285,7 @@
     </row>
     <row r="14" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B14" s="15">
         <v>5726</v>
@@ -1338,7 +1348,7 @@
     </row>
     <row r="16" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="18" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B16" s="6">
         <v>4</v>
@@ -12248,7 +12258,7 @@
         <v>10</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E2" s="8" t="s">
         <v>12</v>
@@ -12290,7 +12300,7 @@
         <v>21</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E3" s="6" t="s">
         <v>71</v>
@@ -12356,7 +12366,7 @@
         <v>76</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>77</v>
@@ -12380,7 +12390,7 @@
         <v>78</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>79</v>
@@ -12404,7 +12414,7 @@
         <v>80</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>81</v>
@@ -12428,7 +12438,7 @@
         <v>82</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>83</v>
@@ -12454,7 +12464,7 @@
         <v>85</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>58</v>
@@ -12601,7 +12611,7 @@
         <v>10</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E16" s="8" t="s">
         <v>99</v>

</xml_diff>

<commit_message>
fix: Handle "Rédactionnel" exposé des motifs
</commit_message>
<xml_diff>
--- a/tests/integration/test_data/test_similarities_expose.xlsx
+++ b/tests/integration/test_data/test_similarities_expose.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10112"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/graal/tests/integration/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6828E34D-8B56-574A-BC39-ABB0D5A17FA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF0C4A61-39B7-6242-94F9-490DB494E81A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="68800" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vieux amendements" sheetId="1" r:id="rId1"/>
@@ -469,7 +469,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -527,6 +527,13 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -561,7 +568,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -615,6 +622,7 @@
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -849,7 +857,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="25" t="s">
         <v>100</v>
       </c>
       <c r="B1" s="16" t="s">

</xml_diff>